<commit_message>
docs: formatted Excel report with semaphores, number formats, and design system
10 sheets with professional formatting:
- Color-coded semaphores: green (CUMPLE/OK), red (NO CUMPLE), amber (PARCIAL)
- Number format: #,##0 for all monetary values
- Frozen panes for header rows
- Tab colors per module
- KPI cards on Resumen sheet
- Monospace font for account codes (Consolas)
- Deducible expenses highlighted in amber
- Acciones de mejora highlighted in red
- Severity badges on Code Review (red=CRITICAL, amber=IMPORTANT)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reporte-validacion-betania.xlsx
+++ b/docs/reporte-validacion-betania.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,8 +52,21 @@
       <color rgb="006B6B6B"/>
       <sz val="9"/>
     </font>
+    <font>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00166534"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -96,8 +109,18 @@
         <bgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -111,11 +134,25 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D4D4D4"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D4D4D4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D4D4D4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D4D4D4"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -136,6 +173,14 @@
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -18566,338 +18611,338 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>Impuesto de Circulación y Tránsito sobre</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Impuesto de Circulación y Tránsito sob</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>1.1.01.02.203</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>1.3.05.59</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr"/>
-      <c r="E5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="11" t="inlineStr"/>
+      <c r="D5" s="16" t="inlineStr"/>
+      <c r="E5" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="16" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Participación en el Impuesto de Vehículo</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Participación en el Impuesto de Vehícu</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>1.1.02.06.003.01.02</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>1.3.05.33</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="7" t="n">
+      <c r="D6" s="18" t="inlineStr"/>
+      <c r="E6" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="19" t="n">
         <v>50873911</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="19" t="n">
         <v>39604652</v>
       </c>
-      <c r="I6" s="7" t="n">
+      <c r="I6" s="19" t="n">
         <v>11269259</v>
       </c>
-      <c r="J6" s="7" t="n">
+      <c r="J6" s="19" t="n">
         <v>0.221513517999432</v>
       </c>
-      <c r="K6" s="7" t="n">
+      <c r="K6" s="19" t="n">
         <v>39604652</v>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="L6" s="20" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Impuesto Predial Unificado</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>1.1.01.01.200</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
         <is>
           <t>1.3.05.07</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr"/>
-      <c r="E7" s="14" t="n">
+      <c r="D7" s="21" t="inlineStr"/>
+      <c r="E7" s="22" t="n">
         <v>2766823305</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="22" t="n">
         <v>902367117.9299999</v>
       </c>
-      <c r="G7" s="14" t="n">
+      <c r="G7" s="22" t="n">
         <v>2369151309.57</v>
       </c>
-      <c r="H7" s="14" t="n">
+      <c r="H7" s="22" t="n">
         <v>1114567886</v>
       </c>
-      <c r="I7" s="14" t="n">
+      <c r="I7" s="22" t="n">
         <v>1254583423.57</v>
       </c>
-      <c r="J7" s="14" t="n">
+      <c r="J7" s="22" t="n">
         <v>0.5295497246217281</v>
       </c>
-      <c r="K7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="15" t="inlineStr">
+      <c r="K7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="23" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Sobretasa Ambiental</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>1.1.01.01.014</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr"/>
-      <c r="D8" s="15" t="inlineStr"/>
-      <c r="E8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="15" t="inlineStr"/>
-      <c r="H8" s="14" t="n">
+      <c r="C8" s="21" t="inlineStr"/>
+      <c r="D8" s="21" t="inlineStr"/>
+      <c r="E8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="21" t="inlineStr"/>
+      <c r="H8" s="22" t="n">
         <v>194805802</v>
       </c>
-      <c r="I8" s="14" t="n">
+      <c r="I8" s="22" t="n">
         <v>-194805802</v>
       </c>
-      <c r="J8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="15" t="inlineStr">
+      <c r="J8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="23" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Impuesto de Industria y Comercio</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>1.1.01.02.200</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>1.3.05.08</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr"/>
-      <c r="E9" s="14" t="n">
+      <c r="D9" s="21" t="inlineStr"/>
+      <c r="E9" s="22" t="n">
         <v>1950044055</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="22" t="n">
         <v>293238596.74</v>
       </c>
-      <c r="G9" s="14" t="n">
+      <c r="G9" s="22" t="n">
         <v>8122489785</v>
       </c>
-      <c r="H9" s="14" t="n">
+      <c r="H9" s="22" t="n">
         <v>453182702</v>
       </c>
-      <c r="I9" s="14" t="n">
+      <c r="I9" s="22" t="n">
         <v>7669307083</v>
       </c>
-      <c r="J9" s="14" t="n">
+      <c r="J9" s="22" t="n">
         <v>0.9442064300484682</v>
       </c>
-      <c r="K9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="15" t="inlineStr">
+      <c r="K9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="23" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>Avisos y Tableros</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>1.1.01.02.201</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>1.3.05.21</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr"/>
-      <c r="E10" s="14" t="n">
+      <c r="D10" s="21" t="inlineStr"/>
+      <c r="E10" s="22" t="n">
         <v>336870699</v>
       </c>
-      <c r="F10" s="14" t="n">
+      <c r="F10" s="22" t="n">
         <v>11927106</v>
       </c>
-      <c r="G10" s="14" t="n">
+      <c r="G10" s="22" t="n">
         <v>850317680</v>
       </c>
-      <c r="H10" s="14" t="n">
+      <c r="H10" s="22" t="n">
         <v>39692416</v>
       </c>
-      <c r="I10" s="14" t="n">
+      <c r="I10" s="22" t="n">
         <v>810625264</v>
       </c>
-      <c r="J10" s="14" t="n">
+      <c r="J10" s="22" t="n">
         <v>0.9533204860564584</v>
       </c>
-      <c r="K10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="15" t="inlineStr">
+      <c r="K10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="23" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Publicidad Exterior Visual</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>1.1.01.02.202</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>1.3.05.58</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr"/>
-      <c r="E11" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="11" t="inlineStr"/>
+      <c r="D11" s="16" t="inlineStr"/>
+      <c r="E11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="16" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Impuesto de Delineación</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>1.1.01.02.204</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>1.3.05.19</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="7" t="n">
+      <c r="D12" s="18" t="inlineStr"/>
+      <c r="E12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="19" t="n">
         <v>97683440</v>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="H12" s="19" t="n">
         <v>84359997</v>
       </c>
-      <c r="I12" s="7" t="n">
+      <c r="I12" s="19" t="n">
         <v>13323443</v>
       </c>
-      <c r="J12" s="7" t="n">
+      <c r="J12" s="19" t="n">
         <v>0.1363940807162402</v>
       </c>
-      <c r="K12" s="7" t="n">
+      <c r="K12" s="19" t="n">
         <v>84359997</v>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="L12" s="20" t="inlineStr">
         <is>
           <t>SI</t>
         </is>

</xml_diff>